<commit_message>
Add Cambodian taxes and full 5-person team to financial model
Model v3: prices treated as VAT-inclusive (10%), 1% profit-tax prepayment,
20% profit tax after loss carry-forward, patent tax, NSSF, and 14%
withholding on foreign services; all 5 team members take the founder
allowance. Update projection, growth and financial-detail drafts and
document how Cambodian tax applies in docs/research.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MF4S689Cu66DaEpymoVfar
</commit_message>
<xml_diff>
--- a/docs/rentify-financial-model.xlsx
+++ b/docs/rentify-financial-model.xlsx
@@ -20,9 +20,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="109">
-  <si>
-    <t xml:space="preserve">Rentify - three-year financial model (bottom-up, v2, Sept 2026)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="120">
+  <si>
+    <t xml:space="preserve">Rentify - three-year financial model (bottom-up, v3, Sept 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Blue = input you can change. Black = formula. Yellow = key assumption to test in the pilot. Years start with the public launch in 2027; the Q4 2026 pilot is covered by Year 1 costs.</t>
@@ -148,16 +148,16 @@
     <t xml:space="preserve">INPUTS - team</t>
   </si>
   <si>
-    <t xml:space="preserve">Full-time founders</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3 full-time founders; the other 2 team members are part-time and paid in equity only.</t>
+    <t xml:space="preserve">Founders (whole team)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All 5 team members hold equity and take the same small allowance.</t>
   </si>
   <si>
     <t xml:space="preserve">Founder allowance ($/founder/month)</t>
   </si>
   <si>
-    <t xml:space="preserve">Founders hold equity, so pay is low: transport and phone in Y1, then a small allowance. Cambodia's 2026 garment minimum wage is $210/month for reference.</t>
+    <t xml:space="preserve">Founders hold equity, so pay is low: transport and phone in Y1, then a small allowance. Cambodia's 2026 garment minimum wage is $210/month for reference. Up to KHR 1.5M (~$375)/month is free of salary tax; above that the employee pays 5%+ (withheld, not a company cost).</t>
   </si>
   <si>
     <t xml:space="preserve">Onboarding/support staff (people)</t>
@@ -172,6 +172,12 @@
     <t xml:space="preserve">Cambodian customer-support roles are reported at about $450-900/month.</t>
   </si>
   <si>
+    <t xml:space="preserve">Employer social security (NSSF, % of pay)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Occupational risk, health care and pension contributions paid by the employer; the pension share rises from 2027. Approximate.</t>
+  </si>
+  <si>
     <t xml:space="preserve">INPUTS - sales and marketing</t>
   </si>
   <si>
@@ -229,22 +235,46 @@
     <t xml:space="preserve">Remote/university space until Year 3 (assumption).</t>
   </si>
   <si>
+    <t xml:space="preserve">VAT-registered (1 = yes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VAT is compulsory above KHR 250M (~$62,500) turnover a year; Rentify passes that in Year 3. A company holding customer payments will likely register from the start, so this is on from Year 1 (conservative).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VAT rate (included in our prices)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10% VAT is charged on sales and passed to the government; it is not a tax on profit. Prices stay $5 incl. VAT, so Rentify keeps $5 / 1.1 = $4.55. VAT we pay on costs can be reclaimed, so costs are shown without VAT.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tax on profit</t>
   </si>
   <si>
-    <t xml:space="preserve">Cambodia standard rate 20%. Losses carried forward.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Minimum tax (% of revenue)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cambodia: 1% of turnover if higher than profit tax. Included to be conservative; startup exemptions may apply.</t>
+    <t xml:space="preserve">20% for companies (medium/large taxpayers). Losses carried forward. IT startups may get a 2-5 year exemption (SME Sub-decree 124, MSME incentives); not assumed here.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prepayment of profit tax (% of revenue)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1% of monthly turnover, credited against profit tax. In loss years it is treated as a cost (conservative). The separate 1% minimum tax does not apply to companies that keep proper accounts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patent tax (annual business tax, $)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KHR 1.2M (~$300) a year for a medium taxpayer. Small enterprises can be exempt for 2 years.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Withholding tax on foreign services</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14% on payments to non-resident suppliers (servers, AI tools, Facebook ads), assumed paid by Rentify on top (conservative).</t>
   </si>
   <si>
     <t xml:space="preserve">Market salary check ($/founder/month)</t>
   </si>
   <si>
-    <t xml:space="preserve">Used only in the sensitivity row: what if founders were paid a typical Phnom Penh developer salary (~$1,000-1,400/month)?</t>
+    <t xml:space="preserve">Used only in the sensitivity row: what if all 5 founders were paid a typical Phnom Penh developer salary (~$1,000-1,400/month)?</t>
   </si>
   <si>
     <t xml:space="preserve">CALCULATIONS</t>
@@ -265,52 +295,55 @@
     <t xml:space="preserve">Sales value of marketplace orders, not Rentify revenue.</t>
   </si>
   <si>
-    <t xml:space="preserve">Infrastructure cost ($/year)</t>
+    <t xml:space="preserve">Infrastructure cost incl. withholding tax ($/year)</t>
   </si>
   <si>
     <t xml:space="preserve">P&amp;L - BASE CASE (subscriptions only)</t>
   </si>
   <si>
+    <t xml:space="preserve">Subscription revenue (excl. VAT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customers pay $5 incl. VAT; the VAT part goes to the government.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost of service (infrastructure)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gross profit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Team (incl. NSSF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sales &amp; marketing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Software, office, legal, patent tax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Result before tax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cumulative result before tax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Higher of the 1% prepayment and 20% profit tax; profit tax only on profit left after earlier losses.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net result</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cumulative net result</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P&amp;L - WITH 3% COMMISSION (upside scenario)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Subscription revenue</t>
   </si>
   <si>
-    <t xml:space="preserve">Cost of service (infrastructure)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gross profit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Team</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sales &amp; marketing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Software, office, legal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Result before tax</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cumulative result before tax</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tax</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Higher of minimum tax and profit tax; profit tax only on profit left after earlier losses.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Net result</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cumulative net result</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P&amp;L - WITH 3% COMMISSION (upside scenario)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Commission revenue</t>
+    <t xml:space="preserve">Commission revenue (excl. VAT)</t>
   </si>
   <si>
     <t xml:space="preserve">Total revenue</t>
@@ -850,7 +883,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E83"/>
+  <dimension ref="A1:E88"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -1213,19 +1246,19 @@
         <v>42</v>
       </c>
       <c r="B27" s="10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C27" s="10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D27" s="10" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E27" s="7" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
         <v>44</v>
       </c>
@@ -1276,38 +1309,38 @@
         <v>49</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B31" s="13" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="C31" s="13" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D31" s="13" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="E31" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C33" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="D33" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="E33" s="3" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="B33" s="16" t="n">
-        <v>100</v>
-      </c>
-      <c r="C33" s="16" t="n">
-        <v>300</v>
-      </c>
-      <c r="D33" s="16" t="n">
-        <v>600</v>
-      </c>
-      <c r="E33" s="7" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1315,13 +1348,13 @@
         <v>53</v>
       </c>
       <c r="B34" s="16" t="n">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="C34" s="16" t="n">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="D34" s="16" t="n">
-        <v>800</v>
+        <v>600</v>
       </c>
       <c r="E34" s="7" t="s">
         <v>54</v>
@@ -1332,13 +1365,13 @@
         <v>55</v>
       </c>
       <c r="B35" s="16" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="C35" s="16" t="n">
         <v>500</v>
       </c>
       <c r="D35" s="16" t="n">
-        <v>1000</v>
+        <v>800</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>56</v>
@@ -1349,13 +1382,13 @@
         <v>57</v>
       </c>
       <c r="B36" s="16" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="C36" s="16" t="n">
-        <v>5</v>
+        <v>500</v>
       </c>
       <c r="D36" s="16" t="n">
-        <v>5</v>
+        <v>1000</v>
       </c>
       <c r="E36" s="7" t="s">
         <v>58</v>
@@ -1365,51 +1398,51 @@
       <c r="A37" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B37" s="13" t="n">
+      <c r="B37" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C37" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="D37" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B38" s="13" t="n">
         <v>0.2</v>
       </c>
-      <c r="C37" s="13" t="n">
+      <c r="C38" s="13" t="n">
         <v>0.2</v>
       </c>
-      <c r="D37" s="13" t="n">
+      <c r="D38" s="13" t="n">
         <v>0.2</v>
       </c>
-      <c r="E37" s="7" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B39" s="4" t="s">
+      <c r="E38" s="7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B40" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="C40" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D39" s="4" t="s">
+      <c r="D40" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E39" s="3" t="s">
+      <c r="E40" s="3" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B40" s="16" t="n">
-        <v>20</v>
-      </c>
-      <c r="C40" s="16" t="n">
-        <v>20</v>
-      </c>
-      <c r="D40" s="16" t="n">
-        <v>20</v>
-      </c>
-      <c r="E40" s="7" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1417,13 +1450,13 @@
         <v>63</v>
       </c>
       <c r="B41" s="16" t="n">
-        <v>840</v>
+        <v>20</v>
       </c>
       <c r="C41" s="16" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="D41" s="16" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E41" s="7" t="s">
         <v>64</v>
@@ -1434,13 +1467,13 @@
         <v>65</v>
       </c>
       <c r="B42" s="16" t="n">
+        <v>840</v>
+      </c>
+      <c r="C42" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="C42" s="16" t="n">
-        <v>50</v>
-      </c>
       <c r="D42" s="16" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="E42" s="7" t="s">
         <v>66</v>
@@ -1454,10 +1487,10 @@
         <v>0</v>
       </c>
       <c r="C43" s="16" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="D43" s="16" t="n">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="E43" s="7" t="s">
         <v>68</v>
@@ -1467,655 +1500,742 @@
       <c r="A44" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B44" s="13" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C44" s="13" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D44" s="13" t="n">
-        <v>0.2</v>
+      <c r="B44" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="16" t="n">
+        <v>150</v>
       </c>
       <c r="E44" s="7" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B45" s="13" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="C45" s="13" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="D45" s="13" t="n">
-        <v>0.01</v>
+      <c r="B45" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="12" t="n">
+        <v>1</v>
       </c>
       <c r="E45" s="7" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="B46" s="16" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C46" s="16" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D46" s="16" t="n">
-        <v>1000</v>
+      <c r="B46" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C46" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D46" s="13" t="n">
+        <v>0.1</v>
       </c>
       <c r="E46" s="7" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="3" t="s">
+    <row r="47" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B48" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D48" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E48" s="3" t="s">
-        <v>6</v>
+      <c r="B47" s="13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C47" s="13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D47" s="13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B48" s="13" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C48" s="13" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D48" s="13" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="E48" s="7" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="B49" s="17" t="n">
+        <v>79</v>
+      </c>
+      <c r="B49" s="16" t="n">
+        <v>300</v>
+      </c>
+      <c r="C49" s="16" t="n">
+        <v>300</v>
+      </c>
+      <c r="D49" s="16" t="n">
+        <v>300</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B50" s="13" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="C50" s="13" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="D50" s="13" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E50" s="7" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B51" s="16" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C51" s="16" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D51" s="16" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E51" s="7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B54" s="17" t="n">
         <f aca="false">B5*B7</f>
         <v>57.6</v>
       </c>
-      <c r="C49" s="17" t="n">
+      <c r="C54" s="17" t="n">
         <f aca="false">C5*C7</f>
         <v>418.85</v>
       </c>
-      <c r="D49" s="17" t="n">
+      <c r="D54" s="17" t="n">
         <f aca="false">D5*D7</f>
         <v>1129.07</v>
       </c>
-      <c r="E49" s="7"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="B50" s="17" t="n">
+      <c r="E54" s="7"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B55" s="17" t="n">
         <f aca="false">B5</f>
         <v>57.6</v>
       </c>
-      <c r="C50" s="17" t="n">
+      <c r="C55" s="17" t="n">
         <f aca="false">C5-B5</f>
         <v>361.25</v>
       </c>
-      <c r="D50" s="17" t="n">
+      <c r="D55" s="17" t="n">
         <f aca="false">D5-C5</f>
         <v>710.22</v>
       </c>
-      <c r="E50" s="7" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B51" s="18" t="n">
-        <f aca="false">(B5+B49)*B11*B12*B13*B10</f>
-        <v>10368</v>
-      </c>
-      <c r="C51" s="18" t="n">
-        <f aca="false">(C5+C49)*C11*C12*C13*C10</f>
-        <v>226179</v>
-      </c>
-      <c r="D51" s="18" t="n">
-        <f aca="false">(D5+D49)*D11*D12*D13*D10</f>
-        <v>812930.4</v>
-      </c>
-      <c r="E51" s="7" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="B52" s="18" t="n">
-        <f aca="false">(B18+B19+B20+B21+B22+B23+B24)*12</f>
-        <v>603</v>
-      </c>
-      <c r="C52" s="18" t="n">
-        <f aca="false">(C18+C19+C20+C21+C22+C23+C24)*12</f>
-        <v>1376.4</v>
-      </c>
-      <c r="D52" s="18" t="n">
-        <f aca="false">(D18+D19+D20+D21+D22+D23+D24)*12</f>
-        <v>2643</v>
-      </c>
-      <c r="E52" s="7"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="B54" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C54" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D54" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E54" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B55" s="18" t="n">
-        <f aca="false">B5*B6*12</f>
-        <v>3456</v>
-      </c>
-      <c r="C55" s="18" t="n">
-        <f aca="false">C5*C6*12</f>
-        <v>25131</v>
-      </c>
-      <c r="D55" s="18" t="n">
-        <f aca="false">D5*D6*12</f>
-        <v>67744.2</v>
-      </c>
-      <c r="E55" s="7"/>
+      <c r="E55" s="7" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B56" s="18" t="n">
-        <f aca="false">B52</f>
-        <v>603</v>
+        <f aca="false">(B5+B54)*B11*B12*B13*B10</f>
+        <v>10368</v>
       </c>
       <c r="C56" s="18" t="n">
-        <f aca="false">C52</f>
-        <v>1376.4</v>
+        <f aca="false">(C5+C54)*C11*C12*C13*C10</f>
+        <v>226179</v>
       </c>
       <c r="D56" s="18" t="n">
-        <f aca="false">D52</f>
-        <v>2643</v>
-      </c>
-      <c r="E56" s="7"/>
+        <f aca="false">(D5+D54)*D11*D12*D13*D10</f>
+        <v>812930.4</v>
+      </c>
+      <c r="E56" s="7" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="19" t="s">
-        <v>85</v>
-      </c>
-      <c r="B57" s="20" t="n">
-        <f aca="false">B55-B56</f>
-        <v>2853</v>
-      </c>
-      <c r="C57" s="20" t="n">
-        <f aca="false">C55-C56</f>
-        <v>23754.6</v>
-      </c>
-      <c r="D57" s="20" t="n">
-        <f aca="false">D55-D56</f>
-        <v>65101.2</v>
+      <c r="A57" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B57" s="18" t="n">
+        <f aca="false">(B18+B19+B20+B21+B22+B23+B24)*12*(1+B50)</f>
+        <v>687.42</v>
+      </c>
+      <c r="C57" s="18" t="n">
+        <f aca="false">(C18+C19+C20+C21+C22+C23+C24)*12*(1+C50)</f>
+        <v>1569.096</v>
+      </c>
+      <c r="D57" s="18" t="n">
+        <f aca="false">(D18+D19+D20+D21+D22+D23+D24)*12*(1+D50)</f>
+        <v>3013.02</v>
       </c>
       <c r="E57" s="7"/>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="B58" s="18" t="n">
-        <f aca="false">B27*B28*12+B29*B30*12</f>
-        <v>3600</v>
-      </c>
-      <c r="C58" s="18" t="n">
-        <f aca="false">C27*C28*12+C29*C30*12</f>
-        <v>10800</v>
-      </c>
-      <c r="D58" s="18" t="n">
-        <f aca="false">D27*D28*12+D29*D30*12</f>
-        <v>24000</v>
-      </c>
-      <c r="E58" s="7"/>
-    </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="B59" s="18" t="n">
-        <f aca="false">B33*12+B34+B35+B50*B37*B36</f>
-        <v>1457.6</v>
-      </c>
-      <c r="C59" s="18" t="n">
-        <f aca="false">C33*12+C34+C35+C50*C37*C36</f>
-        <v>4961.25</v>
-      </c>
-      <c r="D59" s="18" t="n">
-        <f aca="false">D33*12+D34+D35+D50*D37*D36</f>
-        <v>9710.22</v>
-      </c>
-      <c r="E59" s="7"/>
+      <c r="A59" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E59" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B60" s="18" t="n">
-        <f aca="false">B40*B27*12+B41+B42*12+B43*12</f>
-        <v>1560</v>
+        <f aca="false">B5*B6*12/(1+B46*B45)</f>
+        <v>3141.81818181818</v>
       </c>
       <c r="C60" s="18" t="n">
-        <f aca="false">C40*C27*12+C41+C42*12+C43*12</f>
-        <v>1320</v>
+        <f aca="false">C5*C6*12/(1+C46*C45)</f>
+        <v>22846.3636363636</v>
       </c>
       <c r="D60" s="18" t="n">
-        <f aca="false">D40*D27*12+D41+D42*12+D43*12</f>
-        <v>3720</v>
-      </c>
-      <c r="E60" s="7"/>
+        <f aca="false">D5*D6*12/(1+D46*D45)</f>
+        <v>61585.6363636364</v>
+      </c>
+      <c r="E60" s="7" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="19" t="s">
-        <v>89</v>
-      </c>
-      <c r="B61" s="20" t="n">
-        <f aca="false">B57-B58-B59-B60</f>
-        <v>-3764.6</v>
-      </c>
-      <c r="C61" s="20" t="n">
-        <f aca="false">C57-C58-C59-C60</f>
-        <v>6673.35</v>
-      </c>
-      <c r="D61" s="20" t="n">
-        <f aca="false">D57-D58-D59-D60</f>
-        <v>27670.98</v>
+      <c r="A61" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B61" s="18" t="n">
+        <f aca="false">B57</f>
+        <v>687.42</v>
+      </c>
+      <c r="C61" s="18" t="n">
+        <f aca="false">C57</f>
+        <v>1569.096</v>
+      </c>
+      <c r="D61" s="18" t="n">
+        <f aca="false">D57</f>
+        <v>3013.02</v>
       </c>
       <c r="E61" s="7"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="B62" s="18" t="n">
-        <f aca="false">B61</f>
-        <v>-3764.6</v>
-      </c>
-      <c r="C62" s="18" t="n">
-        <f aca="false">B62+C61</f>
-        <v>2908.75</v>
-      </c>
-      <c r="D62" s="18" t="n">
-        <f aca="false">C62+D61</f>
-        <v>30579.73</v>
+      <c r="A62" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="B62" s="20" t="n">
+        <f aca="false">B60-B61</f>
+        <v>2454.39818181818</v>
+      </c>
+      <c r="C62" s="20" t="n">
+        <f aca="false">C60-C61</f>
+        <v>21277.2676363636</v>
+      </c>
+      <c r="D62" s="20" t="n">
+        <f aca="false">D60-D61</f>
+        <v>58572.6163636364</v>
       </c>
       <c r="E62" s="7"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B63" s="18" t="n">
-        <f aca="false">MAX(B45*B55,B44*MAX(0,MIN(B61,B62)))</f>
-        <v>34.56</v>
+        <f aca="false">(B27*B28*12+B29*B30*12)*(1+B31)</f>
+        <v>6360</v>
       </c>
       <c r="C63" s="18" t="n">
-        <f aca="false">MAX(C45*C55,C44*MAX(0,MIN(C61,C62)))</f>
-        <v>581.75</v>
+        <f aca="false">(C27*C28*12+C29*C30*12)*(1+C31)</f>
+        <v>19080</v>
       </c>
       <c r="D63" s="18" t="n">
-        <f aca="false">MAX(D45*D55,D44*MAX(0,MIN(D61,D62)))</f>
-        <v>5534.196</v>
-      </c>
-      <c r="E63" s="7" t="s">
-        <v>92</v>
-      </c>
+        <f aca="false">(D27*D28*12+D29*D30*12)*(1+D31)</f>
+        <v>38520</v>
+      </c>
+      <c r="E63" s="7"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="19" t="s">
-        <v>93</v>
-      </c>
-      <c r="B64" s="20" t="n">
-        <f aca="false">B61-B63</f>
-        <v>-3799.16</v>
-      </c>
-      <c r="C64" s="20" t="n">
-        <f aca="false">C61-C63</f>
-        <v>6091.6</v>
-      </c>
-      <c r="D64" s="20" t="n">
-        <f aca="false">D61-D63</f>
-        <v>22136.784</v>
+      <c r="A64" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="B64" s="18" t="n">
+        <f aca="false">B34*12*(1+B50)+B35+B36+B55*B38*B37</f>
+        <v>1625.6</v>
+      </c>
+      <c r="C64" s="18" t="n">
+        <f aca="false">C34*12*(1+C50)+C35+C36+C55*C38*C37</f>
+        <v>5465.25</v>
+      </c>
+      <c r="D64" s="18" t="n">
+        <f aca="false">D34*12*(1+D50)+D35+D36+D55*D38*D37</f>
+        <v>10718.22</v>
       </c>
       <c r="E64" s="7"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B65" s="18" t="n">
-        <f aca="false">B64</f>
-        <v>-3799.16</v>
+        <f aca="false">B41*B27*12*(1+B50)+B42+B43*12+B44*12+B49</f>
+        <v>2508</v>
       </c>
       <c r="C65" s="18" t="n">
-        <f aca="false">B65+C64</f>
-        <v>2292.44</v>
+        <f aca="false">C41*C27*12*(1+C50)+C42+C43*12+C44*12+C49</f>
+        <v>2268</v>
       </c>
       <c r="D65" s="18" t="n">
-        <f aca="false">C65+D64</f>
-        <v>24429.224</v>
+        <f aca="false">D41*D27*12*(1+D50)+D42+D43*12+D44*12+D49</f>
+        <v>4668</v>
       </c>
       <c r="E65" s="7"/>
     </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="B66" s="20" t="n">
+        <f aca="false">B62-B63-B64-B65</f>
+        <v>-8039.20181818182</v>
+      </c>
+      <c r="C66" s="20" t="n">
+        <f aca="false">C62-C63-C64-C65</f>
+        <v>-5535.98236363637</v>
+      </c>
+      <c r="D66" s="20" t="n">
+        <f aca="false">D62-D63-D64-D65</f>
+        <v>4666.39636363635</v>
+      </c>
+      <c r="E66" s="7"/>
+    </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B67" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C67" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D67" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E67" s="3" t="s">
-        <v>6</v>
-      </c>
+      <c r="A67" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B67" s="18" t="n">
+        <f aca="false">B66</f>
+        <v>-8039.20181818182</v>
+      </c>
+      <c r="C67" s="18" t="n">
+        <f aca="false">B67+C66</f>
+        <v>-13575.1841818182</v>
+      </c>
+      <c r="D67" s="18" t="n">
+        <f aca="false">C67+D66</f>
+        <v>-8908.78781818183</v>
+      </c>
+      <c r="E67" s="7"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="B68" s="18" t="n">
-        <f aca="false">B55</f>
-        <v>3456</v>
+        <f aca="false">MAX(B48*B60,B47*MAX(0,MIN(B66,B67)))</f>
+        <v>31.4181818181818</v>
       </c>
       <c r="C68" s="18" t="n">
-        <f aca="false">C55</f>
-        <v>25131</v>
+        <f aca="false">MAX(C48*C60,C47*MAX(0,MIN(C66,C67)))</f>
+        <v>228.463636363636</v>
       </c>
       <c r="D68" s="18" t="n">
-        <f aca="false">D55</f>
-        <v>67744.2</v>
-      </c>
-      <c r="E68" s="7"/>
+        <f aca="false">MAX(D48*D60,D47*MAX(0,MIN(D66,D67)))</f>
+        <v>615.856363636364</v>
+      </c>
+      <c r="E68" s="7" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="B69" s="18" t="n">
-        <f aca="false">B51*B14</f>
-        <v>311.04</v>
-      </c>
-      <c r="C69" s="18" t="n">
-        <f aca="false">C51*C14</f>
-        <v>6785.37</v>
-      </c>
-      <c r="D69" s="18" t="n">
-        <f aca="false">D51*D14</f>
-        <v>24387.912</v>
+      <c r="A69" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="B69" s="20" t="n">
+        <f aca="false">B66-B68</f>
+        <v>-8070.62</v>
+      </c>
+      <c r="C69" s="20" t="n">
+        <f aca="false">C66-C68</f>
+        <v>-5764.446</v>
+      </c>
+      <c r="D69" s="20" t="n">
+        <f aca="false">D66-D68</f>
+        <v>4050.53999999999</v>
       </c>
       <c r="E69" s="7"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="5" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="B70" s="18" t="n">
-        <f aca="false">B68+B69</f>
-        <v>3767.04</v>
+        <f aca="false">B69</f>
+        <v>-8070.62</v>
       </c>
       <c r="C70" s="18" t="n">
-        <f aca="false">C68+C69</f>
-        <v>31916.37</v>
+        <f aca="false">B70+C69</f>
+        <v>-13835.066</v>
       </c>
       <c r="D70" s="18" t="n">
-        <f aca="false">D68+D69</f>
-        <v>92132.112</v>
+        <f aca="false">C70+D69</f>
+        <v>-9784.52600000002</v>
       </c>
       <c r="E70" s="7"/>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="B71" s="18" t="n">
-        <f aca="false">B52+B51*B15</f>
-        <v>654.84</v>
-      </c>
-      <c r="C71" s="18" t="n">
-        <f aca="false">C52+C51*C15</f>
-        <v>2507.295</v>
-      </c>
-      <c r="D71" s="18" t="n">
-        <f aca="false">D52+D51*D15</f>
-        <v>6707.652</v>
-      </c>
-      <c r="E71" s="7"/>
-    </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="19" t="s">
-        <v>85</v>
-      </c>
-      <c r="B72" s="20" t="n">
-        <f aca="false">B70-B71</f>
-        <v>3112.2</v>
-      </c>
-      <c r="C72" s="20" t="n">
-        <f aca="false">C70-C71</f>
-        <v>29409.075</v>
-      </c>
-      <c r="D72" s="20" t="n">
-        <f aca="false">D70-D71</f>
-        <v>85424.46</v>
-      </c>
-      <c r="E72" s="7"/>
+      <c r="A72" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="5" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="B73" s="18" t="n">
-        <f aca="false">B58+B59+B60</f>
-        <v>6617.6</v>
+        <f aca="false">B60</f>
+        <v>3141.81818181818</v>
       </c>
       <c r="C73" s="18" t="n">
-        <f aca="false">C58+C59+C60</f>
-        <v>17081.25</v>
+        <f aca="false">C60</f>
+        <v>22846.3636363636</v>
       </c>
       <c r="D73" s="18" t="n">
-        <f aca="false">D58+D59+D60</f>
-        <v>37430.22</v>
+        <f aca="false">D60</f>
+        <v>61585.6363636364</v>
       </c>
       <c r="E73" s="7"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="19" t="s">
-        <v>89</v>
-      </c>
-      <c r="B74" s="20" t="n">
-        <f aca="false">B72-B73</f>
-        <v>-3505.4</v>
-      </c>
-      <c r="C74" s="20" t="n">
-        <f aca="false">C72-C73</f>
-        <v>12327.825</v>
-      </c>
-      <c r="D74" s="20" t="n">
-        <f aca="false">D72-D73</f>
-        <v>47994.24</v>
+      <c r="A74" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B74" s="18" t="n">
+        <f aca="false">B56*B14/(1+B46*B45)</f>
+        <v>282.763636363636</v>
+      </c>
+      <c r="C74" s="18" t="n">
+        <f aca="false">C56*C14/(1+C46*C45)</f>
+        <v>6168.51818181818</v>
+      </c>
+      <c r="D74" s="18" t="n">
+        <f aca="false">D56*D14/(1+D46*D45)</f>
+        <v>22170.8290909091</v>
       </c>
       <c r="E74" s="7"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="5" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="B75" s="18" t="n">
-        <f aca="false">B74</f>
-        <v>-3505.4</v>
+        <f aca="false">B73+B74</f>
+        <v>3424.58181818182</v>
       </c>
       <c r="C75" s="18" t="n">
-        <f aca="false">B75+C74</f>
-        <v>8822.425</v>
+        <f aca="false">C73+C74</f>
+        <v>29014.8818181818</v>
       </c>
       <c r="D75" s="18" t="n">
-        <f aca="false">C75+D74</f>
-        <v>56816.665</v>
+        <f aca="false">D73+D74</f>
+        <v>83756.4654545454</v>
       </c>
       <c r="E75" s="7"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="5" t="s">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="B76" s="18" t="n">
-        <f aca="false">MAX(B45*B70,B44*MAX(0,MIN(B74,B75)))</f>
-        <v>37.6704</v>
+        <f aca="false">B57+B56*B15</f>
+        <v>739.26</v>
       </c>
       <c r="C76" s="18" t="n">
-        <f aca="false">MAX(C45*C70,C44*MAX(0,MIN(C74,C75)))</f>
-        <v>1764.485</v>
+        <f aca="false">C57+C56*C15</f>
+        <v>2699.991</v>
       </c>
       <c r="D76" s="18" t="n">
-        <f aca="false">MAX(D45*D70,D44*MAX(0,MIN(D74,D75)))</f>
-        <v>9598.848</v>
+        <f aca="false">D57+D56*D15</f>
+        <v>7077.672</v>
       </c>
       <c r="E76" s="7"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="19" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B77" s="20" t="n">
-        <f aca="false">B74-B76</f>
-        <v>-3543.0704</v>
+        <f aca="false">B75-B76</f>
+        <v>2685.32181818182</v>
       </c>
       <c r="C77" s="20" t="n">
-        <f aca="false">C74-C76</f>
-        <v>10563.34</v>
+        <f aca="false">C75-C76</f>
+        <v>26314.8908181818</v>
       </c>
       <c r="D77" s="20" t="n">
-        <f aca="false">D74-D76</f>
-        <v>38395.392</v>
+        <f aca="false">D75-D76</f>
+        <v>76678.7934545454</v>
       </c>
       <c r="E77" s="7"/>
     </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B78" s="18" t="n">
+        <f aca="false">B63+B64+B65</f>
+        <v>10493.6</v>
+      </c>
+      <c r="C78" s="18" t="n">
+        <f aca="false">C63+C64+C65</f>
+        <v>26813.25</v>
+      </c>
+      <c r="D78" s="18" t="n">
+        <f aca="false">D63+D64+D65</f>
+        <v>53906.22</v>
+      </c>
+      <c r="E78" s="7"/>
+    </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="3" t="s">
+      <c r="A79" s="19" t="s">
         <v>100</v>
       </c>
-      <c r="B79" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C79" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D79" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E79" s="3" t="s">
-        <v>6</v>
-      </c>
+      <c r="B79" s="20" t="n">
+        <f aca="false">B77-B78</f>
+        <v>-7808.27818181818</v>
+      </c>
+      <c r="C79" s="20" t="n">
+        <f aca="false">C77-C78</f>
+        <v>-498.359181818181</v>
+      </c>
+      <c r="D79" s="20" t="n">
+        <f aca="false">D77-D78</f>
+        <v>22772.5734545454</v>
+      </c>
+      <c r="E79" s="7"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B80" s="21" t="n">
-        <f aca="false">(B58+B59+B60+B56)/(B6*12)</f>
-        <v>120.343333333333</v>
-      </c>
-      <c r="C80" s="21" t="n">
-        <f aca="false">(C58+C59+C60+C56)/(C6*12)</f>
-        <v>307.6275</v>
-      </c>
-      <c r="D80" s="21" t="n">
-        <f aca="false">(D58+D59+D60+D56)/(D6*12)</f>
-        <v>667.887</v>
-      </c>
-      <c r="E80" s="7" t="s">
-        <v>102</v>
-      </c>
+      <c r="B80" s="18" t="n">
+        <f aca="false">B79</f>
+        <v>-7808.27818181818</v>
+      </c>
+      <c r="C80" s="18" t="n">
+        <f aca="false">B80+C79</f>
+        <v>-8306.63736363636</v>
+      </c>
+      <c r="D80" s="18" t="n">
+        <f aca="false">C80+D79</f>
+        <v>14465.9360909091</v>
+      </c>
+      <c r="E80" s="7"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B81" s="18" t="n">
+        <f aca="false">MAX(B48*B75,B47*MAX(0,MIN(B79,B80)))</f>
+        <v>34.2458181818182</v>
+      </c>
+      <c r="C81" s="18" t="n">
+        <f aca="false">MAX(C48*C75,C47*MAX(0,MIN(C79,C80)))</f>
+        <v>290.148818181818</v>
+      </c>
+      <c r="D81" s="18" t="n">
+        <f aca="false">MAX(D48*D75,D47*MAX(0,MIN(D79,D80)))</f>
+        <v>2893.18721818181</v>
+      </c>
+      <c r="E81" s="7"/>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="B81" s="22" t="n">
-        <f aca="false">B80/65433</f>
-        <v>0.00183918410180388</v>
-      </c>
-      <c r="C81" s="22" t="n">
-        <f aca="false">C80/65433</f>
-        <v>0.00470141213149328</v>
-      </c>
-      <c r="D81" s="22" t="n">
-        <f aca="false">D80/65433</f>
-        <v>0.0102071890330567</v>
-      </c>
-      <c r="E81" s="7" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="B82" s="18" t="n">
-        <f aca="false">-MIN(0,MIN($B$65:B65))</f>
-        <v>3799.16</v>
-      </c>
-      <c r="C82" s="18" t="n">
-        <f aca="false">-MIN(0,MIN($B$65:C65))</f>
-        <v>3799.16</v>
-      </c>
-      <c r="D82" s="18" t="n">
-        <f aca="false">-MIN(0,MIN($B$65:D65))</f>
-        <v>3799.16</v>
-      </c>
-      <c r="E82" s="7" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A83" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="B83" s="18" t="n">
-        <f aca="false">B64-B27*(B46-B28)*12*(1-IF(B61&gt;0,B44,0))</f>
-        <v>-36199.16</v>
-      </c>
-      <c r="C83" s="18" t="n">
-        <f aca="false">C64-C27*(C46-C28)*12*(1-IF(C61&gt;0,C44,0))</f>
-        <v>-14068.4</v>
-      </c>
-      <c r="D83" s="18" t="n">
-        <f aca="false">D64-D27*(D46-D28)*12*(1-IF(D61&gt;0,D44,0))</f>
-        <v>7736.784</v>
-      </c>
-      <c r="E83" s="7" t="s">
-        <v>108</v>
+      <c r="B82" s="20" t="n">
+        <f aca="false">B79-B81</f>
+        <v>-7842.524</v>
+      </c>
+      <c r="C82" s="20" t="n">
+        <f aca="false">C79-C81</f>
+        <v>-788.508</v>
+      </c>
+      <c r="D82" s="20" t="n">
+        <f aca="false">D79-D81</f>
+        <v>19879.3862363636</v>
+      </c>
+      <c r="E82" s="7"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D84" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E84" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B85" s="21" t="n">
+        <f aca="false">(B63+B64+B65+B61)/(B6*12/(1+B46*B45))</f>
+        <v>204.985366666667</v>
+      </c>
+      <c r="C85" s="21" t="n">
+        <f aca="false">(C63+C64+C65+C61)/(C6*12/(1+C46*C45))</f>
+        <v>520.34301</v>
+      </c>
+      <c r="D85" s="21" t="n">
+        <f aca="false">(D63+D64+D65+D61)/(D6*12/(1+D46*D45))</f>
+        <v>1043.5194</v>
+      </c>
+      <c r="E85" s="7" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B86" s="22" t="n">
+        <f aca="false">B85/65433</f>
+        <v>0.00313275207718837</v>
+      </c>
+      <c r="C86" s="22" t="n">
+        <f aca="false">C85/65433</f>
+        <v>0.00795230250790885</v>
+      </c>
+      <c r="D86" s="22" t="n">
+        <f aca="false">D85/65433</f>
+        <v>0.0159479070193939</v>
+      </c>
+      <c r="E86" s="7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="B87" s="18" t="n">
+        <f aca="false">-MIN(0,MIN($B$70:B70))</f>
+        <v>8070.62</v>
+      </c>
+      <c r="C87" s="18" t="n">
+        <f aca="false">-MIN(0,MIN($B$70:C70))</f>
+        <v>13835.066</v>
+      </c>
+      <c r="D87" s="18" t="n">
+        <f aca="false">-MIN(0,MIN($B$70:D70))</f>
+        <v>13835.066</v>
+      </c>
+      <c r="E87" s="7" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="B88" s="18" t="n">
+        <f aca="false">B69-B27*(B51-B28)*12*(1+B31)*(1-IF(B66&gt;0,B47,0))</f>
+        <v>-65310.62</v>
+      </c>
+      <c r="C88" s="18" t="n">
+        <f aca="false">C69-C27*(C51-C28)*12*(1+C31)*(1-IF(C66&gt;0,C47,0))</f>
+        <v>-50284.446</v>
+      </c>
+      <c r="D88" s="18" t="n">
+        <f aca="false">D69-D27*(D51-D28)*12*(1+D31)*(1-IF(D66&gt;0,D47,0))</f>
+        <v>-21629.46</v>
+      </c>
+      <c r="E88" s="7" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rework financial model for a bootstrapped five-person team
Model v4: the team is unpaid in Year 1, then takes half of each year's
profit (max $500 per founder a month); marketing is 10% of revenue plus
referral credits; shared AI tools, no office rent, no hires, accountant
from Year 3. Projection slide now shows where each year's revenue goes.
Add bootstrapped benchmarks and caveats to docs/research.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MF4S689Cu66DaEpymoVfar
</commit_message>
<xml_diff>
--- a/docs/rentify-financial-model.xlsx
+++ b/docs/rentify-financial-model.xlsx
@@ -20,9 +20,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="120">
-  <si>
-    <t xml:space="preserve">Rentify - three-year financial model (bottom-up, v3, Sept 2026)</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="123">
+  <si>
+    <t xml:space="preserve">Rentify - three-year financial model (bootstrapped, v4, Sept 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Blue = input you can change. Black = formula. Yellow = key assumption to test in the pilot. Years start with the public launch in 2027; the Q4 2026 pilot is covered by Year 1 costs.</t>
@@ -145,94 +145,91 @@
     <t xml:space="preserve">About $15/year. SSL is free (Let's Encrypt). Merchants buy their own custom domains.</t>
   </si>
   <si>
-    <t xml:space="preserve">INPUTS - team</t>
+    <t xml:space="preserve">INPUTS - team (paid from profit)</t>
   </si>
   <si>
     <t xml:space="preserve">Founders (whole team)</t>
   </si>
   <si>
-    <t xml:space="preserve">All 5 team members hold equity and take the same small allowance.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Founder allowance ($/founder/month)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Founders hold equity, so pay is low: transport and phone in Y1, then a small allowance. Cambodia's 2026 garment minimum wage is $210/month for reference. Up to KHR 1.5M (~$375)/month is free of salary tax; above that the employee pays 5%+ (withheld, not a company cost).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Onboarding/support staff (people)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Founders do onboarding and support until Year 3.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Staff salary ($/month)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cambodian customer-support roles are reported at about $450-900/month.</t>
+    <t xml:space="preserve">All 5 team members hold equity and do everything themselves: product, sales, onboarding, support. No hires in Years 1-3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of profit paid to the team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bootstrapped rule: the team works unpaid until there is profit, then takes half of each year's profit (before team pay) and keeps the other half as reserve. Many bootstrapped founders start at $0 and stay under ~$1,000/month for years (Pilot founder salary report; Practical Founders).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maximum pay per founder ($/month)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cap, so extra profit is reinvested. Up to KHR 1.5M (~$375)/month is free of salary tax; above that the employee pays 5% (withheld, not a company cost).</t>
   </si>
   <si>
     <t xml:space="preserve">Employer social security (NSSF, % of pay)</t>
   </si>
   <si>
-    <t xml:space="preserve">Occupational risk, health care and pension contributions paid by the employer; the pension share rises from 2027. Approximate.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">INPUTS - sales and marketing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Facebook ads ($/month)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Assumption: small targeted budget that grows with the business.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Printed QR stands and flyers ($/year)</t>
+    <t xml:space="preserve">Occupational risk, health care and pension contributions paid by the employer on team pay; the pension share rises from 2027. Approximate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INPUTS - sales and marketing (limited budget)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Marketing budget (% of revenue)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spend only what revenue allows: ads, printed QR stands, festival campaigns. Growth is founder-led (shop visits, Facebook groups, referrals), so this sits below the 20-40% that early bootstrapped SaaS firms often spend on marketing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimum launch materials ($/year)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Printed QR stands and flyers for the first pilot shops, before revenue exists.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referral credit per referred paying shop ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One month free for the shop that refers another.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share of new paying shops that come by referral</t>
   </si>
   <si>
     <t xml:space="preserve">Assumption.</t>
   </si>
   <si>
-    <t xml:space="preserve">Festival and category campaigns ($/year)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Assumption, e.g. Khmer New Year campaigns.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Referral credit per referred paying shop ($)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One month free for the shop that refers another.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Share of new paying shops that come by referral</t>
-  </si>
-  <si>
     <t xml:space="preserve">INPUTS - software, office, legal and tax</t>
   </si>
   <si>
-    <t xml:space="preserve">AI tools ($/founder/month)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claude Pro or ChatGPT Plus, about $20/month each. Code hosting (GitHub) and design tools use free plans.</t>
+    <t xml:space="preserve">Shared AI tool subscriptions (number)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The team shares a few accounts instead of one each.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI tool price ($/subscription/month)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Claude Pro or ChatGPT Plus, about $20/month. Code hosting (GitHub) and design tools use free plans.</t>
   </si>
   <si>
     <t xml:space="preserve">Company registration (one-off)</t>
   </si>
   <si>
-    <t xml:space="preserve">Ministry of Commerce fee about KHR 2,155,000 (~$540) plus ~$300 notary/legal help. Year 1 only.</t>
+    <t xml:space="preserve">Ministry of Commerce fee about KHR 2,155,000 (~$540) plus ~$300 notary/legal help. Needed before online payments (2027).</t>
   </si>
   <si>
     <t xml:space="preserve">Bookkeeping and tax filing ($/month)</t>
   </si>
   <si>
-    <t xml:space="preserve">Founders in Y1; outsourced accountant from Y2 (assumption).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coworking desk ($/month)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Remote/university space until Year 3 (assumption).</t>
+    <t xml:space="preserve">Founders keep the books in Years 1-2; a part-time accountant from Year 3 (proper records also avoid the 1% minimum tax).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Office ($/month)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No rent: home, university, or free startup space such as Techo Startup Center in Phnom Penh.</t>
   </si>
   <si>
     <t xml:space="preserve">VAT-registered (1 = yes)</t>
@@ -268,13 +265,7 @@
     <t xml:space="preserve">Withholding tax on foreign services</t>
   </si>
   <si>
-    <t xml:space="preserve">14% on payments to non-resident suppliers (servers, AI tools, Facebook ads), assumed paid by Rentify on top (conservative).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Market salary check ($/founder/month)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Used only in the sensitivity row: what if all 5 founders were paid a typical Phnom Penh developer salary (~$1,000-1,400/month)?</t>
+    <t xml:space="preserve">14% on payments to non-resident suppliers (servers, AI tools), assumed paid by Rentify on top (conservative).</t>
   </si>
   <si>
     <t xml:space="preserve">CALCULATIONS</t>
@@ -298,6 +289,15 @@
     <t xml:space="preserve">Infrastructure cost incl. withholding tax ($/year)</t>
   </si>
   <si>
+    <t xml:space="preserve">Subscription Rentify keeps per shop ($/year, excl. VAT)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Software, office, legal, patent tax ($/year)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Team pay cap ($/year)</t>
+  </si>
+  <si>
     <t xml:space="preserve">P&amp;L - BASE CASE (subscriptions only)</t>
   </si>
   <si>
@@ -313,15 +313,24 @@
     <t xml:space="preserve">Gross profit</t>
   </si>
   <si>
-    <t xml:space="preserve">Team (incl. NSSF)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sales &amp; marketing</t>
   </si>
   <si>
     <t xml:space="preserve">Software, office, legal, patent tax</t>
   </si>
   <si>
+    <t xml:space="preserve">Profit before team pay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What the business earns while the team works for equity.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Team pay (from profit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Team cost incl. NSSF</t>
+  </si>
+  <si>
     <t xml:space="preserve">Result before tax</t>
   </si>
   <si>
@@ -331,12 +340,15 @@
     <t xml:space="preserve">Higher of the 1% prepayment and 20% profit tax; profit tax only on profit left after earlier losses.</t>
   </si>
   <si>
-    <t xml:space="preserve">Net result</t>
+    <t xml:space="preserve">Net result (kept in the company)</t>
   </si>
   <si>
     <t xml:space="preserve">Cumulative net result</t>
   </si>
   <si>
+    <t xml:space="preserve">Pay per founder ($/month)</t>
+  </si>
+  <si>
     <t xml:space="preserve">P&amp;L - WITH 3% COMMISSION (upside scenario)</t>
   </si>
   <si>
@@ -352,34 +364,31 @@
     <t xml:space="preserve">Cost of service (infrastructure + payment cost)</t>
   </si>
   <si>
-    <t xml:space="preserve">Operating costs (same as base)</t>
-  </si>
-  <si>
     <t xml:space="preserve">KEY FIGURES</t>
   </si>
   <si>
-    <t xml:space="preserve">Break-even paying shops (base case, that year's costs)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yearly fixed costs / yearly subscription per shop. Infrastructure is treated as fixed at this scale.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Break-even as share of SAM (65,433 stores)</t>
+    <t xml:space="preserve">Paying shops needed to cover running costs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Costs excluding team pay / what each paying shop leaves after marketing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paying shops needed to also pay every founder the cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shows when all 5 founders could take the full monthly cap.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">...as share of SAM (65,433 stores)</t>
   </si>
   <si>
     <t xml:space="preserve">NIS Economic Census 2022, ISIC 4741-4774.</t>
   </si>
   <si>
-    <t xml:space="preserve">Funding needed (largest cumulative loss, base case)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cash the team must raise (prize money, grants, savings) before profits cover costs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sensitivity: net result if founders earned market salary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Approximate: base-case net result with founder pay raised to the market-salary check. Shows the model does not depend on unpaid work forever.</t>
+    <t xml:space="preserve">Cash needed before first revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registration, launch materials and about 3 months of servers during the pilot; from savings or prize money.</t>
   </si>
 </sst>
 </file>
@@ -599,10 +608,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="170" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -612,6 +617,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -883,7 +892,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E88"/>
+  <dimension ref="A1:E95"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -1262,99 +1271,99 @@
       <c r="A28" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="B28" s="15" t="n">
-        <v>100</v>
-      </c>
-      <c r="C28" s="15" t="n">
-        <v>300</v>
-      </c>
-      <c r="D28" s="15" t="n">
-        <v>500</v>
+      <c r="B28" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="11" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D28" s="11" t="n">
+        <v>0.5</v>
       </c>
       <c r="E28" s="7" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B29" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="C29" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" s="10" t="n">
-        <v>1</v>
+      <c r="B29" s="15" t="n">
+        <v>500</v>
+      </c>
+      <c r="C29" s="15" t="n">
+        <v>500</v>
+      </c>
+      <c r="D29" s="15" t="n">
+        <v>500</v>
       </c>
       <c r="E29" s="7" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B30" s="16" t="n">
-        <v>500</v>
-      </c>
-      <c r="C30" s="16" t="n">
-        <v>500</v>
-      </c>
-      <c r="D30" s="16" t="n">
-        <v>500</v>
+      <c r="B30" s="13" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="C30" s="13" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D30" s="13" t="n">
+        <v>0.07</v>
       </c>
       <c r="E30" s="7" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B31" s="13" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="C31" s="13" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="D31" s="13" t="n">
-        <v>0.07</v>
-      </c>
-      <c r="E31" s="7" t="s">
+      <c r="B32" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
+      <c r="B33" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C33" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D33" s="11" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E33" s="7" t="s">
         <v>52</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B34" s="16" t="n">
+      <c r="B34" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="C34" s="16" t="n">
-        <v>300</v>
-      </c>
-      <c r="D34" s="16" t="n">
-        <v>600</v>
+      <c r="C34" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="15" t="n">
+        <v>0</v>
       </c>
       <c r="E34" s="7" t="s">
         <v>54</v>
@@ -1364,14 +1373,14 @@
       <c r="A35" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B35" s="16" t="n">
-        <v>200</v>
-      </c>
-      <c r="C35" s="16" t="n">
-        <v>500</v>
-      </c>
-      <c r="D35" s="16" t="n">
-        <v>800</v>
+      <c r="B35" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C35" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="D35" s="15" t="n">
+        <v>5</v>
       </c>
       <c r="E35" s="7" t="s">
         <v>56</v>
@@ -1381,272 +1390,276 @@
       <c r="A36" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="B36" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="C36" s="16" t="n">
-        <v>500</v>
-      </c>
-      <c r="D36" s="16" t="n">
-        <v>1000</v>
+      <c r="B36" s="13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C36" s="13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D36" s="13" t="n">
+        <v>0.2</v>
       </c>
       <c r="E36" s="7" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5" t="s">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B37" s="16" t="n">
+      <c r="B38" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D38" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C37" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="D37" s="16" t="n">
-        <v>5</v>
-      </c>
-      <c r="E37" s="7" t="s">
+      <c r="E38" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="5" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5" t="s">
+      <c r="B39" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C39" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D39" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E39" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B38" s="13" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C38" s="13" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D38" s="13" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E38" s="7" t="s">
-        <v>56</v>
-      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="s">
+      <c r="A40" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B40" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E40" s="3" t="s">
-        <v>6</v>
+      <c r="B40" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="C40" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="D40" s="15" t="n">
+        <v>20</v>
+      </c>
+      <c r="E40" s="7" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="B41" s="16" t="n">
-        <v>20</v>
-      </c>
-      <c r="C41" s="16" t="n">
-        <v>20</v>
-      </c>
-      <c r="D41" s="16" t="n">
-        <v>20</v>
+        <v>64</v>
+      </c>
+      <c r="B41" s="15" t="n">
+        <v>840</v>
+      </c>
+      <c r="C41" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" s="15" t="n">
+        <v>0</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="B42" s="16" t="n">
-        <v>840</v>
-      </c>
-      <c r="C42" s="16" t="n">
+        <v>66</v>
+      </c>
+      <c r="B42" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="D42" s="16" t="n">
+      <c r="C42" s="15" t="n">
         <v>0</v>
       </c>
+      <c r="D42" s="15" t="n">
+        <v>50</v>
+      </c>
       <c r="E42" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B43" s="16" t="n">
+        <v>68</v>
+      </c>
+      <c r="B43" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="C43" s="16" t="n">
-        <v>50</v>
-      </c>
-      <c r="D43" s="16" t="n">
-        <v>100</v>
+      <c r="C43" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" s="15" t="n">
+        <v>0</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="B44" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="C44" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D44" s="16" t="n">
-        <v>150</v>
+        <v>70</v>
+      </c>
+      <c r="B44" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D44" s="12" t="n">
+        <v>1</v>
       </c>
       <c r="E44" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B45" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C45" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" s="12" t="n">
-        <v>1</v>
+        <v>72</v>
+      </c>
+      <c r="B45" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C45" s="13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D45" s="13" t="n">
+        <v>0.1</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B46" s="13" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="C46" s="13" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="D46" s="13" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="E46" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B47" s="13" t="n">
-        <v>0.2</v>
+        <v>0.01</v>
       </c>
       <c r="C47" s="13" t="n">
-        <v>0.2</v>
+        <v>0.01</v>
       </c>
       <c r="D47" s="13" t="n">
-        <v>0.2</v>
+        <v>0.01</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="B48" s="13" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="C48" s="13" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="D48" s="13" t="n">
-        <v>0.01</v>
+        <v>78</v>
+      </c>
+      <c r="B48" s="15" t="n">
+        <v>300</v>
+      </c>
+      <c r="C48" s="15" t="n">
+        <v>300</v>
+      </c>
+      <c r="D48" s="15" t="n">
+        <v>300</v>
       </c>
       <c r="E48" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B49" s="16" t="n">
-        <v>300</v>
-      </c>
-      <c r="C49" s="16" t="n">
-        <v>300</v>
-      </c>
-      <c r="D49" s="16" t="n">
-        <v>300</v>
+        <v>80</v>
+      </c>
+      <c r="B49" s="13" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="C49" s="13" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="D49" s="13" t="n">
+        <v>0.14</v>
       </c>
       <c r="E49" s="7" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="B50" s="13" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="C50" s="13" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="D50" s="13" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="E50" s="7" t="s">
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="3" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="5" t="s">
+      <c r="B51" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E51" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="B51" s="16" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C51" s="16" t="n">
-        <v>1000</v>
-      </c>
-      <c r="D51" s="16" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E51" s="7" t="s">
+      <c r="B52" s="16" t="n">
+        <f aca="false">B5*B7</f>
+        <v>57.6</v>
+      </c>
+      <c r="C52" s="16" t="n">
+        <f aca="false">C5*C7</f>
+        <v>418.85</v>
+      </c>
+      <c r="D52" s="16" t="n">
+        <f aca="false">D5*D7</f>
+        <v>1129.07</v>
+      </c>
+      <c r="E52" s="7"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="5" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="3" t="s">
+      <c r="B53" s="16" t="n">
+        <f aca="false">B5</f>
+        <v>57.6</v>
+      </c>
+      <c r="C53" s="16" t="n">
+        <f aca="false">C5-B5</f>
+        <v>361.25</v>
+      </c>
+      <c r="D53" s="16" t="n">
+        <f aca="false">D5-C5</f>
+        <v>710.22</v>
+      </c>
+      <c r="E53" s="7" t="s">
         <v>85</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D53" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E53" s="3" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1654,259 +1667,257 @@
         <v>86</v>
       </c>
       <c r="B54" s="17" t="n">
-        <f aca="false">B5*B7</f>
-        <v>57.6</v>
+        <f aca="false">(B5+B52)*B11*B12*B13*B10</f>
+        <v>10368</v>
       </c>
       <c r="C54" s="17" t="n">
-        <f aca="false">C5*C7</f>
-        <v>418.85</v>
+        <f aca="false">(C5+C52)*C11*C12*C13*C10</f>
+        <v>226179</v>
       </c>
       <c r="D54" s="17" t="n">
-        <f aca="false">D5*D7</f>
-        <v>1129.07</v>
-      </c>
-      <c r="E54" s="7"/>
+        <f aca="false">(D5+D52)*D11*D12*D13*D10</f>
+        <v>812930.4</v>
+      </c>
+      <c r="E54" s="7" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B55" s="17" t="n">
-        <f aca="false">B5</f>
-        <v>57.6</v>
+        <f aca="false">(B18+B19+B20+B21+B22+B23+B24)*12*(1+B49)</f>
+        <v>687.42</v>
       </c>
       <c r="C55" s="17" t="n">
-        <f aca="false">C5-B5</f>
-        <v>361.25</v>
+        <f aca="false">(C18+C19+C20+C21+C22+C23+C24)*12*(1+C49)</f>
+        <v>1569.096</v>
       </c>
       <c r="D55" s="17" t="n">
-        <f aca="false">D5-C5</f>
-        <v>710.22</v>
-      </c>
-      <c r="E55" s="7" t="s">
-        <v>88</v>
-      </c>
+        <f aca="false">(D18+D19+D20+D21+D22+D23+D24)*12*(1+D49)</f>
+        <v>3013.02</v>
+      </c>
+      <c r="E55" s="7"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="5" t="s">
         <v>89</v>
       </c>
       <c r="B56" s="18" t="n">
-        <f aca="false">(B5+B54)*B11*B12*B13*B10</f>
-        <v>10368</v>
+        <f aca="false">B6*12/(1+B45*B44)</f>
+        <v>54.5454545454545</v>
       </c>
       <c r="C56" s="18" t="n">
-        <f aca="false">(C5+C54)*C11*C12*C13*C10</f>
-        <v>226179</v>
+        <f aca="false">C6*12/(1+C45*C44)</f>
+        <v>54.5454545454545</v>
       </c>
       <c r="D56" s="18" t="n">
-        <f aca="false">(D5+D54)*D11*D12*D13*D10</f>
-        <v>812930.4</v>
-      </c>
-      <c r="E56" s="7" t="s">
-        <v>90</v>
-      </c>
+        <f aca="false">D6*12/(1+D45*D44)</f>
+        <v>54.5454545454545</v>
+      </c>
+      <c r="E56" s="7"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B57" s="17" t="n">
+        <f aca="false">B39*B40*12*(1+B49)+B41+B42*12+B43*12+B48</f>
+        <v>1687.2</v>
+      </c>
+      <c r="C57" s="17" t="n">
+        <f aca="false">C39*C40*12*(1+C49)+C41+C42*12+C43*12+C48</f>
+        <v>847.2</v>
+      </c>
+      <c r="D57" s="17" t="n">
+        <f aca="false">D39*D40*12*(1+D49)+D41+D42*12+D43*12+D48</f>
+        <v>1720.8</v>
+      </c>
+      <c r="E57" s="7"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B57" s="18" t="n">
-        <f aca="false">(B18+B19+B20+B21+B22+B23+B24)*12*(1+B50)</f>
-        <v>687.42</v>
-      </c>
-      <c r="C57" s="18" t="n">
-        <f aca="false">(C18+C19+C20+C21+C22+C23+C24)*12*(1+C50)</f>
-        <v>1569.096</v>
-      </c>
-      <c r="D57" s="18" t="n">
-        <f aca="false">(D18+D19+D20+D21+D22+D23+D24)*12*(1+D50)</f>
-        <v>3013.02</v>
-      </c>
-      <c r="E57" s="7"/>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="3" t="s">
+      <c r="B58" s="17" t="n">
+        <f aca="false">B27*B29*12</f>
+        <v>30000</v>
+      </c>
+      <c r="C58" s="17" t="n">
+        <f aca="false">C27*C29*12</f>
+        <v>30000</v>
+      </c>
+      <c r="D58" s="17" t="n">
+        <f aca="false">D27*D29*12</f>
+        <v>30000</v>
+      </c>
+      <c r="E58" s="7"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B59" s="4" t="s">
+      <c r="B60" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C59" s="4" t="s">
+      <c r="C60" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D59" s="4" t="s">
+      <c r="D60" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E59" s="3" t="s">
+      <c r="E60" s="3" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B60" s="18" t="n">
-        <f aca="false">B5*B6*12/(1+B46*B45)</f>
-        <v>3141.81818181818</v>
-      </c>
-      <c r="C60" s="18" t="n">
-        <f aca="false">C5*C6*12/(1+C46*C45)</f>
-        <v>22846.3636363636</v>
-      </c>
-      <c r="D60" s="18" t="n">
-        <f aca="false">D5*D6*12/(1+D46*D45)</f>
-        <v>61585.6363636364</v>
-      </c>
-      <c r="E60" s="7" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="B61" s="17" t="n">
+        <f aca="false">B5*B56</f>
+        <v>3141.81818181818</v>
+      </c>
+      <c r="C61" s="17" t="n">
+        <f aca="false">C5*C56</f>
+        <v>22846.3636363636</v>
+      </c>
+      <c r="D61" s="17" t="n">
+        <f aca="false">D5*D56</f>
+        <v>61585.6363636364</v>
+      </c>
+      <c r="E61" s="7" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="B61" s="18" t="n">
-        <f aca="false">B57</f>
+      <c r="B62" s="17" t="n">
+        <f aca="false">B55</f>
         <v>687.42</v>
       </c>
-      <c r="C61" s="18" t="n">
-        <f aca="false">C57</f>
+      <c r="C62" s="17" t="n">
+        <f aca="false">C55</f>
         <v>1569.096</v>
       </c>
-      <c r="D61" s="18" t="n">
-        <f aca="false">D57</f>
+      <c r="D62" s="17" t="n">
+        <f aca="false">D55</f>
         <v>3013.02</v>
       </c>
-      <c r="E61" s="7"/>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="19" t="s">
+      <c r="E62" s="7"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="B62" s="20" t="n">
-        <f aca="false">B60-B61</f>
+      <c r="B63" s="20" t="n">
+        <f aca="false">B61-B62</f>
         <v>2454.39818181818</v>
       </c>
-      <c r="C62" s="20" t="n">
-        <f aca="false">C60-C61</f>
+      <c r="C63" s="20" t="n">
+        <f aca="false">C61-C62</f>
         <v>21277.2676363636</v>
       </c>
-      <c r="D62" s="20" t="n">
-        <f aca="false">D60-D61</f>
+      <c r="D63" s="20" t="n">
+        <f aca="false">D61-D62</f>
         <v>58572.6163636364</v>
-      </c>
-      <c r="E62" s="7"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="B63" s="18" t="n">
-        <f aca="false">(B27*B28*12+B29*B30*12)*(1+B31)</f>
-        <v>6360</v>
-      </c>
-      <c r="C63" s="18" t="n">
-        <f aca="false">(C27*C28*12+C29*C30*12)*(1+C31)</f>
-        <v>19080</v>
-      </c>
-      <c r="D63" s="18" t="n">
-        <f aca="false">(D27*D28*12+D29*D30*12)*(1+D31)</f>
-        <v>38520</v>
       </c>
       <c r="E63" s="7"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="B64" s="18" t="n">
-        <f aca="false">B34*12*(1+B50)+B35+B36+B55*B38*B37</f>
-        <v>1625.6</v>
-      </c>
-      <c r="C64" s="18" t="n">
-        <f aca="false">C34*12*(1+C50)+C35+C36+C55*C38*C37</f>
-        <v>5465.25</v>
-      </c>
-      <c r="D64" s="18" t="n">
-        <f aca="false">D34*12*(1+D50)+D35+D36+D55*D38*D37</f>
-        <v>10718.22</v>
+        <v>97</v>
+      </c>
+      <c r="B64" s="17" t="n">
+        <f aca="false">B33*B61+B34+B53*B36*B35</f>
+        <v>471.781818181818</v>
+      </c>
+      <c r="C64" s="17" t="n">
+        <f aca="false">C33*C61+C34+C53*C36*C35</f>
+        <v>2645.88636363636</v>
+      </c>
+      <c r="D64" s="17" t="n">
+        <f aca="false">D33*D61+D34+D53*D36*D35</f>
+        <v>6868.78363636364</v>
       </c>
       <c r="E64" s="7"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="B65" s="18" t="n">
-        <f aca="false">B41*B27*12*(1+B50)+B42+B43*12+B44*12+B49</f>
-        <v>2508</v>
-      </c>
-      <c r="C65" s="18" t="n">
-        <f aca="false">C41*C27*12*(1+C50)+C42+C43*12+C44*12+C49</f>
-        <v>2268</v>
-      </c>
-      <c r="D65" s="18" t="n">
-        <f aca="false">D41*D27*12*(1+D50)+D42+D43*12+D44*12+D49</f>
-        <v>4668</v>
+        <v>98</v>
+      </c>
+      <c r="B65" s="17" t="n">
+        <f aca="false">B57</f>
+        <v>1687.2</v>
+      </c>
+      <c r="C65" s="17" t="n">
+        <f aca="false">C57</f>
+        <v>847.2</v>
+      </c>
+      <c r="D65" s="17" t="n">
+        <f aca="false">D57</f>
+        <v>1720.8</v>
       </c>
       <c r="E65" s="7"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="B66" s="20" t="n">
+        <f aca="false">B63-B64-B65</f>
+        <v>295.416363636363</v>
+      </c>
+      <c r="C66" s="20" t="n">
+        <f aca="false">C63-C64-C65</f>
+        <v>17784.1812727273</v>
+      </c>
+      <c r="D66" s="20" t="n">
+        <f aca="false">D63-D64-D65</f>
+        <v>49983.0327272727</v>
+      </c>
+      <c r="E66" s="7" t="s">
         <v>100</v>
       </c>
-      <c r="B66" s="20" t="n">
-        <f aca="false">B62-B63-B64-B65</f>
-        <v>-8039.20181818182</v>
-      </c>
-      <c r="C66" s="20" t="n">
-        <f aca="false">C62-C63-C64-C65</f>
-        <v>-5535.98236363637</v>
-      </c>
-      <c r="D66" s="20" t="n">
-        <f aca="false">D62-D63-D64-D65</f>
-        <v>4666.39636363635</v>
-      </c>
-      <c r="E66" s="7"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B67" s="18" t="n">
-        <f aca="false">B66</f>
-        <v>-8039.20181818182</v>
-      </c>
-      <c r="C67" s="18" t="n">
-        <f aca="false">B67+C66</f>
-        <v>-13575.1841818182</v>
-      </c>
-      <c r="D67" s="18" t="n">
-        <f aca="false">C67+D66</f>
-        <v>-8908.78781818183</v>
+      <c r="B67" s="17" t="n">
+        <f aca="false">MIN(B58,B28*MAX(0,B66))</f>
+        <v>0</v>
+      </c>
+      <c r="C67" s="17" t="n">
+        <f aca="false">MIN(C58,C28*MAX(0,C66))</f>
+        <v>8892.09063636364</v>
+      </c>
+      <c r="D67" s="17" t="n">
+        <f aca="false">MIN(D58,D28*MAX(0,D66))</f>
+        <v>24991.5163636364</v>
       </c>
       <c r="E67" s="7"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B68" s="18" t="n">
-        <f aca="false">MAX(B48*B60,B47*MAX(0,MIN(B66,B67)))</f>
-        <v>31.4181818181818</v>
-      </c>
-      <c r="C68" s="18" t="n">
-        <f aca="false">MAX(C48*C60,C47*MAX(0,MIN(C66,C67)))</f>
-        <v>228.463636363636</v>
-      </c>
-      <c r="D68" s="18" t="n">
-        <f aca="false">MAX(D48*D60,D47*MAX(0,MIN(D66,D67)))</f>
-        <v>615.856363636364</v>
-      </c>
-      <c r="E68" s="7" t="s">
         <v>102</v>
       </c>
+      <c r="B68" s="17" t="n">
+        <f aca="false">B67*(1+B30)</f>
+        <v>0</v>
+      </c>
+      <c r="C68" s="17" t="n">
+        <f aca="false">C67*(1+C30)</f>
+        <v>9425.61607454545</v>
+      </c>
+      <c r="D68" s="17" t="n">
+        <f aca="false">D67*(1+D30)</f>
+        <v>26740.9225090909</v>
+      </c>
+      <c r="E68" s="7"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="19" t="s">
@@ -1914,15 +1925,15 @@
       </c>
       <c r="B69" s="20" t="n">
         <f aca="false">B66-B68</f>
-        <v>-8070.62</v>
+        <v>295.416363636363</v>
       </c>
       <c r="C69" s="20" t="n">
         <f aca="false">C66-C68</f>
-        <v>-5764.446</v>
+        <v>8358.56519818182</v>
       </c>
       <c r="D69" s="20" t="n">
         <f aca="false">D66-D68</f>
-        <v>4050.53999999999</v>
+        <v>23242.1102181818</v>
       </c>
       <c r="E69" s="7"/>
     </row>
@@ -1930,312 +1941,440 @@
       <c r="A70" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="B70" s="18" t="n">
+      <c r="B70" s="17" t="n">
         <f aca="false">B69</f>
-        <v>-8070.62</v>
-      </c>
-      <c r="C70" s="18" t="n">
+        <v>295.416363636363</v>
+      </c>
+      <c r="C70" s="17" t="n">
         <f aca="false">B70+C69</f>
-        <v>-13835.066</v>
-      </c>
-      <c r="D70" s="18" t="n">
+        <v>8653.98156181818</v>
+      </c>
+      <c r="D70" s="17" t="n">
         <f aca="false">C70+D69</f>
-        <v>-9784.52600000002</v>
+        <v>31896.09178</v>
       </c>
       <c r="E70" s="7"/>
     </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B71" s="17" t="n">
+        <f aca="false">MAX(B47*B61,B46*MAX(0,MIN(B69,B70)))</f>
+        <v>59.0832727272727</v>
+      </c>
+      <c r="C71" s="17" t="n">
+        <f aca="false">MAX(C47*C61,C46*MAX(0,MIN(C69,C70)))</f>
+        <v>1671.71303963636</v>
+      </c>
+      <c r="D71" s="17" t="n">
+        <f aca="false">MAX(D47*D61,D46*MAX(0,MIN(D69,D70)))</f>
+        <v>4648.42204363636</v>
+      </c>
+      <c r="E71" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="B72" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C72" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D72" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E72" s="3" t="s">
-        <v>6</v>
-      </c>
+      <c r="A72" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="B72" s="20" t="n">
+        <f aca="false">B69-B71</f>
+        <v>236.333090909091</v>
+      </c>
+      <c r="C72" s="20" t="n">
+        <f aca="false">C69-C71</f>
+        <v>6686.85215854545</v>
+      </c>
+      <c r="D72" s="20" t="n">
+        <f aca="false">D69-D71</f>
+        <v>18593.6881745454</v>
+      </c>
+      <c r="E72" s="7"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="B73" s="18" t="n">
-        <f aca="false">B60</f>
+        <v>107</v>
+      </c>
+      <c r="B73" s="17" t="n">
+        <f aca="false">B72</f>
+        <v>236.333090909091</v>
+      </c>
+      <c r="C73" s="17" t="n">
+        <f aca="false">B73+C72</f>
+        <v>6923.18524945454</v>
+      </c>
+      <c r="D73" s="17" t="n">
+        <f aca="false">C73+D72</f>
+        <v>25516.873424</v>
+      </c>
+      <c r="E73" s="7"/>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="B74" s="20" t="n">
+        <f aca="false">B67/B27/12</f>
+        <v>0</v>
+      </c>
+      <c r="C74" s="20" t="n">
+        <f aca="false">C67/C27/12</f>
+        <v>148.201510606061</v>
+      </c>
+      <c r="D74" s="20" t="n">
+        <f aca="false">D67/D27/12</f>
+        <v>416.525272727273</v>
+      </c>
+      <c r="E74" s="7"/>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E76" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="B77" s="17" t="n">
+        <f aca="false">B61</f>
         <v>3141.81818181818</v>
       </c>
-      <c r="C73" s="18" t="n">
-        <f aca="false">C60</f>
+      <c r="C77" s="17" t="n">
+        <f aca="false">C61</f>
         <v>22846.3636363636</v>
       </c>
-      <c r="D73" s="18" t="n">
-        <f aca="false">D60</f>
+      <c r="D77" s="17" t="n">
+        <f aca="false">D61</f>
         <v>61585.6363636364</v>
-      </c>
-      <c r="E73" s="7"/>
-    </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A74" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="B74" s="18" t="n">
-        <f aca="false">B56*B14/(1+B46*B45)</f>
-        <v>282.763636363636</v>
-      </c>
-      <c r="C74" s="18" t="n">
-        <f aca="false">C56*C14/(1+C46*C45)</f>
-        <v>6168.51818181818</v>
-      </c>
-      <c r="D74" s="18" t="n">
-        <f aca="false">D56*D14/(1+D46*D45)</f>
-        <v>22170.8290909091</v>
-      </c>
-      <c r="E74" s="7"/>
-    </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="B75" s="18" t="n">
-        <f aca="false">B73+B74</f>
-        <v>3424.58181818182</v>
-      </c>
-      <c r="C75" s="18" t="n">
-        <f aca="false">C73+C74</f>
-        <v>29014.8818181818</v>
-      </c>
-      <c r="D75" s="18" t="n">
-        <f aca="false">D73+D74</f>
-        <v>83756.4654545454</v>
-      </c>
-      <c r="E75" s="7"/>
-    </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A76" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="B76" s="18" t="n">
-        <f aca="false">B57+B56*B15</f>
-        <v>739.26</v>
-      </c>
-      <c r="C76" s="18" t="n">
-        <f aca="false">C57+C56*C15</f>
-        <v>2699.991</v>
-      </c>
-      <c r="D76" s="18" t="n">
-        <f aca="false">D57+D56*D15</f>
-        <v>7077.672</v>
-      </c>
-      <c r="E76" s="7"/>
-    </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="19" t="s">
-        <v>96</v>
-      </c>
-      <c r="B77" s="20" t="n">
-        <f aca="false">B75-B76</f>
-        <v>2685.32181818182</v>
-      </c>
-      <c r="C77" s="20" t="n">
-        <f aca="false">C75-C76</f>
-        <v>26314.8908181818</v>
-      </c>
-      <c r="D77" s="20" t="n">
-        <f aca="false">D75-D76</f>
-        <v>76678.7934545454</v>
       </c>
       <c r="E77" s="7"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="B78" s="18" t="n">
-        <f aca="false">B63+B64+B65</f>
-        <v>10493.6</v>
-      </c>
-      <c r="C78" s="18" t="n">
-        <f aca="false">C63+C64+C65</f>
-        <v>26813.25</v>
-      </c>
-      <c r="D78" s="18" t="n">
-        <f aca="false">D63+D64+D65</f>
-        <v>53906.22</v>
+        <v>111</v>
+      </c>
+      <c r="B78" s="17" t="n">
+        <f aca="false">B54*B14/(1+B45*B44)</f>
+        <v>282.763636363636</v>
+      </c>
+      <c r="C78" s="17" t="n">
+        <f aca="false">C54*C14/(1+C45*C44)</f>
+        <v>6168.51818181818</v>
+      </c>
+      <c r="D78" s="17" t="n">
+        <f aca="false">D54*D14/(1+D45*D44)</f>
+        <v>22170.8290909091</v>
       </c>
       <c r="E78" s="7"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="19" t="s">
-        <v>100</v>
-      </c>
-      <c r="B79" s="20" t="n">
-        <f aca="false">B77-B78</f>
-        <v>-7808.27818181818</v>
-      </c>
-      <c r="C79" s="20" t="n">
-        <f aca="false">C77-C78</f>
-        <v>-498.359181818181</v>
-      </c>
-      <c r="D79" s="20" t="n">
-        <f aca="false">D77-D78</f>
-        <v>22772.5734545454</v>
+      <c r="A79" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B79" s="17" t="n">
+        <f aca="false">B77+B78</f>
+        <v>3424.58181818182</v>
+      </c>
+      <c r="C79" s="17" t="n">
+        <f aca="false">C77+C78</f>
+        <v>29014.8818181818</v>
+      </c>
+      <c r="D79" s="17" t="n">
+        <f aca="false">D77+D78</f>
+        <v>83756.4654545454</v>
       </c>
       <c r="E79" s="7"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B80" s="17" t="n">
+        <f aca="false">B55+B54*B15</f>
+        <v>739.26</v>
+      </c>
+      <c r="C80" s="17" t="n">
+        <f aca="false">C55+C54*C15</f>
+        <v>2699.991</v>
+      </c>
+      <c r="D80" s="17" t="n">
+        <f aca="false">D55+D54*D15</f>
+        <v>7077.672</v>
+      </c>
+      <c r="E80" s="7"/>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="B81" s="20" t="n">
+        <f aca="false">B79-B80</f>
+        <v>2685.32181818182</v>
+      </c>
+      <c r="C81" s="20" t="n">
+        <f aca="false">C79-C80</f>
+        <v>26314.8908181818</v>
+      </c>
+      <c r="D81" s="20" t="n">
+        <f aca="false">D79-D80</f>
+        <v>76678.7934545454</v>
+      </c>
+      <c r="E81" s="7"/>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B82" s="17" t="n">
+        <f aca="false">B33*B79+B34+B53*B36*B35</f>
+        <v>500.058181818182</v>
+      </c>
+      <c r="C82" s="17" t="n">
+        <f aca="false">C33*C79+C34+C53*C36*C35</f>
+        <v>3262.73818181818</v>
+      </c>
+      <c r="D82" s="17" t="n">
+        <f aca="false">D33*D79+D34+D53*D36*D35</f>
+        <v>9085.86654545454</v>
+      </c>
+      <c r="E82" s="7"/>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="B83" s="20" t="n">
+        <f aca="false">B81-B82-B57</f>
+        <v>498.063636363636</v>
+      </c>
+      <c r="C83" s="20" t="n">
+        <f aca="false">C81-C82-C57</f>
+        <v>22204.9526363636</v>
+      </c>
+      <c r="D83" s="20" t="n">
+        <f aca="false">D81-D82-D57</f>
+        <v>65872.1269090909</v>
+      </c>
+      <c r="E83" s="7"/>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B80" s="18" t="n">
-        <f aca="false">B79</f>
-        <v>-7808.27818181818</v>
-      </c>
-      <c r="C80" s="18" t="n">
-        <f aca="false">B80+C79</f>
-        <v>-8306.63736363636</v>
-      </c>
-      <c r="D80" s="18" t="n">
-        <f aca="false">C80+D79</f>
-        <v>14465.9360909091</v>
-      </c>
-      <c r="E80" s="7"/>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B81" s="18" t="n">
-        <f aca="false">MAX(B48*B75,B47*MAX(0,MIN(B79,B80)))</f>
-        <v>34.2458181818182</v>
-      </c>
-      <c r="C81" s="18" t="n">
-        <f aca="false">MAX(C48*C75,C47*MAX(0,MIN(C79,C80)))</f>
-        <v>290.148818181818</v>
-      </c>
-      <c r="D81" s="18" t="n">
-        <f aca="false">MAX(D48*D75,D47*MAX(0,MIN(D79,D80)))</f>
-        <v>2893.18721818181</v>
-      </c>
-      <c r="E81" s="7"/>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="19" t="s">
+      <c r="B84" s="17" t="n">
+        <f aca="false">MIN(B58,B28*MAX(0,B83))</f>
+        <v>0</v>
+      </c>
+      <c r="C84" s="17" t="n">
+        <f aca="false">MIN(C58,C28*MAX(0,C83))</f>
+        <v>11102.4763181818</v>
+      </c>
+      <c r="D84" s="17" t="n">
+        <f aca="false">MIN(D58,D28*MAX(0,D83))</f>
+        <v>30000</v>
+      </c>
+      <c r="E84" s="7"/>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="19" t="s">
         <v>103</v>
       </c>
-      <c r="B82" s="20" t="n">
-        <f aca="false">B79-B81</f>
-        <v>-7842.524</v>
-      </c>
-      <c r="C82" s="20" t="n">
-        <f aca="false">C79-C81</f>
-        <v>-788.508</v>
-      </c>
-      <c r="D82" s="20" t="n">
-        <f aca="false">D79-D81</f>
-        <v>19879.3862363636</v>
-      </c>
-      <c r="E82" s="7"/>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A84" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="B84" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C84" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="D84" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E84" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="B85" s="21" t="n">
-        <f aca="false">(B63+B64+B65+B61)/(B6*12/(1+B46*B45))</f>
-        <v>204.985366666667</v>
-      </c>
-      <c r="C85" s="21" t="n">
-        <f aca="false">(C63+C64+C65+C61)/(C6*12/(1+C46*C45))</f>
-        <v>520.34301</v>
-      </c>
-      <c r="D85" s="21" t="n">
-        <f aca="false">(D63+D64+D65+D61)/(D6*12/(1+D46*D45))</f>
-        <v>1043.5194</v>
-      </c>
-      <c r="E85" s="7" t="s">
-        <v>113</v>
-      </c>
+      <c r="B85" s="20" t="n">
+        <f aca="false">B83-B84*(1+B30)</f>
+        <v>498.063636363636</v>
+      </c>
+      <c r="C85" s="20" t="n">
+        <f aca="false">C83-C84*(1+C30)</f>
+        <v>10436.3277390909</v>
+      </c>
+      <c r="D85" s="20" t="n">
+        <f aca="false">D83-D84*(1+D30)</f>
+        <v>33772.1269090909</v>
+      </c>
+      <c r="E85" s="7"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="B86" s="22" t="n">
-        <f aca="false">B85/65433</f>
-        <v>0.00313275207718837</v>
-      </c>
-      <c r="C86" s="22" t="n">
-        <f aca="false">C85/65433</f>
-        <v>0.00795230250790885</v>
-      </c>
-      <c r="D86" s="22" t="n">
-        <f aca="false">D85/65433</f>
-        <v>0.0159479070193939</v>
-      </c>
-      <c r="E86" s="7" t="s">
-        <v>115</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="B86" s="17" t="n">
+        <f aca="false">B85</f>
+        <v>498.063636363636</v>
+      </c>
+      <c r="C86" s="17" t="n">
+        <f aca="false">B86+C85</f>
+        <v>10934.3913754545</v>
+      </c>
+      <c r="D86" s="17" t="n">
+        <f aca="false">C86+D85</f>
+        <v>44706.5182845454</v>
+      </c>
+      <c r="E86" s="7"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="B87" s="17" t="n">
+        <f aca="false">MAX(B47*B79,B46*MAX(0,MIN(B85,B86)))</f>
+        <v>99.6127272727271</v>
+      </c>
+      <c r="C87" s="17" t="n">
+        <f aca="false">MAX(C47*C79,C46*MAX(0,MIN(C85,C86)))</f>
+        <v>2087.26554781818</v>
+      </c>
+      <c r="D87" s="17" t="n">
+        <f aca="false">MAX(D47*D79,D46*MAX(0,MIN(D85,D86)))</f>
+        <v>6754.42538181818</v>
+      </c>
+      <c r="E87" s="7"/>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="B88" s="20" t="n">
+        <f aca="false">B85-B87</f>
+        <v>398.450909090909</v>
+      </c>
+      <c r="C88" s="20" t="n">
+        <f aca="false">C85-C87</f>
+        <v>8349.06219127273</v>
+      </c>
+      <c r="D88" s="20" t="n">
+        <f aca="false">D85-D87</f>
+        <v>27017.7015272727</v>
+      </c>
+      <c r="E88" s="7"/>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="B89" s="20" t="n">
+        <f aca="false">B84/B27/12</f>
+        <v>0</v>
+      </c>
+      <c r="C89" s="20" t="n">
+        <f aca="false">C84/C27/12</f>
+        <v>185.041271969697</v>
+      </c>
+      <c r="D89" s="20" t="n">
+        <f aca="false">D84/D27/12</f>
+        <v>500</v>
+      </c>
+      <c r="E89" s="7"/>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D91" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E91" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B92" s="21" t="n">
+        <f aca="false">(B62+B57+B34+B53*B36*B35)/(B56*(1-B33))</f>
+        <v>51.5822592592593</v>
+      </c>
+      <c r="C92" s="21" t="n">
+        <f aca="false">(C62+C57+C34+C53*C36*C35)/(C56*(1-C33))</f>
+        <v>56.5796407407408</v>
+      </c>
+      <c r="D92" s="21" t="n">
+        <f aca="false">(D62+D57+D34+D53*D36*D35)/(D56*(1-D33))</f>
+        <v>110.897111111111</v>
+      </c>
+      <c r="E92" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="B87" s="18" t="n">
-        <f aca="false">-MIN(0,MIN($B$70:B70))</f>
-        <v>8070.62</v>
-      </c>
-      <c r="C87" s="18" t="n">
-        <f aca="false">-MIN(0,MIN($B$70:C70))</f>
-        <v>13835.066</v>
-      </c>
-      <c r="D87" s="18" t="n">
-        <f aca="false">-MIN(0,MIN($B$70:D70))</f>
-        <v>13835.066</v>
-      </c>
-      <c r="E87" s="7" t="s">
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="5" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="88" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="5" t="s">
+      <c r="B93" s="21" t="n">
+        <f aca="false">(B62+B57+B34+B53*B36*B35+B58*(1+B30))/(B56*(1-B33))</f>
+        <v>699.360037037037</v>
+      </c>
+      <c r="C93" s="21" t="n">
+        <f aca="false">(C62+C57+C34+C53*C36*C35+C58*(1+C30))/(C56*(1-C33))</f>
+        <v>704.357418518519</v>
+      </c>
+      <c r="D93" s="21" t="n">
+        <f aca="false">(D62+D57+D34+D53*D36*D35+D58*(1+D30))/(D56*(1-D33))</f>
+        <v>764.786</v>
+      </c>
+      <c r="E93" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="B88" s="18" t="n">
-        <f aca="false">B69-B27*(B51-B28)*12*(1+B31)*(1-IF(B66&gt;0,B47,0))</f>
-        <v>-65310.62</v>
-      </c>
-      <c r="C88" s="18" t="n">
-        <f aca="false">C69-C27*(C51-C28)*12*(1+C31)*(1-IF(C66&gt;0,C47,0))</f>
-        <v>-50284.446</v>
-      </c>
-      <c r="D88" s="18" t="n">
-        <f aca="false">D69-D27*(D51-D28)*12*(1+D31)*(1-IF(D66&gt;0,D47,0))</f>
-        <v>-21629.46</v>
-      </c>
-      <c r="E88" s="7" t="s">
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="5" t="s">
         <v>119</v>
+      </c>
+      <c r="B94" s="22" t="n">
+        <f aca="false">B93/65433</f>
+        <v>0.01068818542688</v>
+      </c>
+      <c r="C94" s="22" t="n">
+        <f aca="false">C93/65433</f>
+        <v>0.0107645594504076</v>
+      </c>
+      <c r="D94" s="22" t="n">
+        <f aca="false">D93/65433</f>
+        <v>0.0116880778811915</v>
+      </c>
+      <c r="E94" s="7" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B95" s="17" t="n">
+        <f aca="false">B41+B34+B55/4</f>
+        <v>1111.855</v>
+      </c>
+      <c r="C95" s="17" t="n">
+        <f aca="false">0</f>
+        <v>0</v>
+      </c>
+      <c r="D95" s="17" t="n">
+        <f aca="false">0</f>
+        <v>0</v>
+      </c>
+      <c r="E95" s="7" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>